<commit_message>
feat(facturare): add Qty column to proforma template and PDF
- Add qty field to OrderLine model (default 1)
- Parse qty from column I in proforma Anexa
- Display actual qty in collapsed PDF table
- Update Anexa_Proforma_Template.xlsx with Qty column

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/jarvis/accounting/facturare/assets/Anexa_Proforma_Template.xlsx
+++ b/jarvis/accounting/facturare/assets/Anexa_Proforma_Template.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -487,6 +487,11 @@
           <t>Invoice Date</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -524,6 +529,9 @@
         <is>
           <t>2026-04-30</t>
         </is>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>